<commit_message>
refactor: split STW pipeline into step scripts
</commit_message>
<xml_diff>
--- a/STW programs/STW_sitefile_and_mapping.xlsx
+++ b/STW programs/STW_sitefile_and_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/finnfujimura/Desktop/LEI-SRML-Intern-Project/STW programs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\finnf\Desktop\LEI-SRML-Intern-Project\STW programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9144FD34-92E7-E647-BA79-D60AC4971DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76A56CF-80F2-4854-A879-D9BD9079E865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31230" yWindow="1740" windowWidth="22230" windowHeight="12930" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="STW site" sheetId="2" r:id="rId1"/>
@@ -1791,6 +1791,7 @@
     <xf numFmtId="0" fontId="22" fillId="48" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="47" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="47" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="48" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1803,7 +1804,6 @@
     <xf numFmtId="0" fontId="16" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="48" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -5154,42 +5154,42 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V185"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="4.83203125" style="17" customWidth="1"/>
-    <col min="8" max="9" width="18.6640625" style="43" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" style="43" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="4.85546875" style="17" customWidth="1"/>
+    <col min="8" max="9" width="18.7109375" style="43" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" style="43" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="3" style="15" customWidth="1"/>
-    <col min="12" max="12" width="23.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="22.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="4.33203125" style="17" customWidth="1"/>
-    <col min="16" max="16" width="22.33203125" style="43" customWidth="1"/>
+    <col min="12" max="12" width="23.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="4.28515625" style="17" customWidth="1"/>
+    <col min="16" max="16" width="22.28515625" style="43" customWidth="1"/>
     <col min="17" max="17" width="33" style="43" customWidth="1"/>
-    <col min="18" max="18" width="47.83203125" style="43" customWidth="1"/>
-    <col min="19" max="19" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="47.85546875" style="43" customWidth="1"/>
+    <col min="19" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
-      <c r="D1" s="76" t="s">
+      <c r="D1" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="76"/>
-      <c r="F1" s="78" t="s">
+      <c r="E1" s="77"/>
+      <c r="F1" s="79" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="79"/>
-      <c r="H1" s="77" t="s">
+      <c r="G1" s="80"/>
+      <c r="H1" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I1" s="77"/>
+      <c r="I1" s="78"/>
       <c r="J1" s="46"/>
       <c r="K1" s="13"/>
       <c r="L1" s="5" t="s">
@@ -5214,7 +5214,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -5238,7 +5238,7 @@
       <c r="U2"/>
       <c r="V2"/>
     </row>
-    <row r="3" spans="1:22" ht="48" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" ht="45" x14ac:dyDescent="0.25">
       <c r="D3" s="3" t="s">
         <v>0</v>
       </c>
@@ -5262,7 +5262,7 @@
       </c>
       <c r="K3" s="14"/>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="D4" s="4" t="s">
         <v>114</v>
       </c>
@@ -5290,7 +5290,7 @@
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="1:22" ht="96" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -5331,7 +5331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -5345,7 +5345,7 @@
       <c r="I6" s="42"/>
       <c r="J6" s="42"/>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
@@ -5359,7 +5359,7 @@
       <c r="I7" s="42"/>
       <c r="J7" s="42"/>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
@@ -5373,7 +5373,7 @@
       <c r="I8" s="42"/>
       <c r="J8" s="42"/>
     </row>
-    <row r="9" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
@@ -5397,7 +5397,7 @@
       <c r="Q9" s="43"/>
       <c r="R9" s="42"/>
     </row>
-    <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
@@ -5439,7 +5439,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="C11" s="9"/>
     </row>
-    <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -5457,12 +5457,12 @@
       </c>
       <c r="C12" s="9"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="10">
         <f>IF(LEN(C14)=17,LEFT(C14,4)+(B14-1)/(DATE(LEFT(C14,4)+1,1,1)-DATE(LEFT(C14,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2015.7478310502283</v>
@@ -5481,7 +5481,7 @@
       <c r="P14" s="48"/>
       <c r="Q14" s="48"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="16">
         <v>1000</v>
       </c>
@@ -5536,7 +5536,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>2010</v>
       </c>
@@ -5591,7 +5591,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>9300</v>
       </c>
@@ -5645,12 +5645,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="21">
         <f>IF(LEN(C19)=17,LEFT(C19,4)+(B19-1)/(DATE(LEFT(C19,4)+1,1,1)-DATE(LEFT(C19,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2016.0000018973892</v>
@@ -5669,7 +5669,7 @@
       <c r="P19" s="48"/>
       <c r="Q19" s="48"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="16">
         <v>1000</v>
       </c>
@@ -5724,7 +5724,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>2010</v>
       </c>
@@ -5779,7 +5779,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>9300</v>
       </c>
@@ -5833,12 +5833,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="20">
         <f>IF(LEN(C24)=17,LEFT(C24,4)+(B24-1)/(DATE(LEFT(C24,4)+1,1,1)-DATE(LEFT(C24,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2017.0000019025874</v>
@@ -5857,7 +5857,7 @@
       <c r="P24" s="48"/>
       <c r="Q24" s="48"/>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="16">
         <v>1000</v>
       </c>
@@ -5912,7 +5912,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>2010</v>
       </c>
@@ -5967,7 +5967,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>9300</v>
       </c>
@@ -6021,12 +6021,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="10">
         <f>IF(LEN(C29)=17,LEFT(C29,4)+(B29-1)/(DATE(LEFT(C29,4)+1,1,1)-DATE(LEFT(C29,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2017.5821537290715</v>
@@ -6045,7 +6045,7 @@
       <c r="P29" s="48"/>
       <c r="Q29" s="48"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="16">
         <v>1000</v>
       </c>
@@ -6100,7 +6100,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>2010</v>
       </c>
@@ -6155,7 +6155,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>9300</v>
       </c>
@@ -6209,12 +6209,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" s="10">
         <f>IF(LEN(C34)=17,LEFT(C34,4)+(B34-1)/(DATE(LEFT(C34,4)+1,1,1)-DATE(LEFT(C34,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2018.0000019025874</v>
@@ -6233,7 +6233,7 @@
       <c r="P34" s="48"/>
       <c r="Q34" s="48"/>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" s="16">
         <v>1000</v>
       </c>
@@ -6288,7 +6288,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>2010</v>
       </c>
@@ -6343,7 +6343,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>9300</v>
       </c>
@@ -6397,12 +6397,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" s="10">
         <f>IF(LEN(C39)=17,LEFT(C39,4)+(B39-1)/(DATE(LEFT(C39,4)+1,1,1)-DATE(LEFT(C39,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2019.0000019025874</v>
@@ -6421,7 +6421,7 @@
       <c r="P39" s="48"/>
       <c r="Q39" s="48"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" s="16">
         <v>1000</v>
       </c>
@@ -6476,7 +6476,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>2010</v>
       </c>
@@ -6531,7 +6531,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>9300</v>
       </c>
@@ -6585,12 +6585,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" s="10">
         <f>IF(LEN(C44)=17,LEFT(C44,4)+(B44-1)/(DATE(LEFT(C44,4)+1,1,1)-DATE(LEFT(C44,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2020.0000018973892</v>
@@ -6609,7 +6609,7 @@
       <c r="P44" s="48"/>
       <c r="Q44" s="48"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="16">
         <v>1000</v>
       </c>
@@ -6664,7 +6664,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>2010</v>
       </c>
@@ -6719,7 +6719,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>9300</v>
       </c>
@@ -6773,7 +6773,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>0</v>
       </c>
@@ -6826,12 +6826,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A50" s="10">
         <f>IF(LEN(C50)=17,LEFT(C50,4)+(B50-1)/(DATE(LEFT(C50,4)+1,1,1)-DATE(LEFT(C50,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2020.5819691105039</v>
@@ -6853,7 +6853,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A51" s="16">
         <v>1000</v>
       </c>
@@ -6909,7 +6909,7 @@
       </c>
       <c r="S51" s="28"/>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A52" s="16">
         <v>2010</v>
       </c>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="S52" s="28"/>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A53" s="16">
         <v>3000</v>
       </c>
@@ -7021,7 +7021,7 @@
       </c>
       <c r="S53" s="28"/>
     </row>
-    <row r="54" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A54" s="16">
         <v>0</v>
       </c>
@@ -7077,7 +7077,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="55" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A55" s="16">
         <v>0</v>
       </c>
@@ -7136,7 +7136,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="56" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A56" s="16">
         <v>0</v>
       </c>
@@ -7195,7 +7195,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>78</v>
       </c>
@@ -7250,7 +7250,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>79</v>
       </c>
@@ -7305,7 +7305,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A59" s="10" t="s">
         <v>80</v>
       </c>
@@ -7360,7 +7360,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>7009</v>
       </c>
@@ -7416,7 +7416,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>7008</v>
       </c>
@@ -7469,7 +7469,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>9388</v>
       </c>
@@ -7522,7 +7522,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>9389</v>
       </c>
@@ -7575,7 +7575,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>9300</v>
       </c>
@@ -7629,7 +7629,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>0</v>
       </c>
@@ -7682,12 +7682,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A67" s="10">
         <f>IF(LEN(C67)=17,LEFT(C67,4)+(B67-1)/(DATE(LEFT(C67,4)+1,1,1)-DATE(LEFT(C67,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2021.0000019025874</v>
@@ -7709,7 +7709,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A68" s="16">
         <v>1000</v>
       </c>
@@ -7765,7 +7765,7 @@
       </c>
       <c r="S68" s="28"/>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A69" s="16">
         <v>2010</v>
       </c>
@@ -7821,7 +7821,7 @@
       </c>
       <c r="S69" s="28"/>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A70" s="16">
         <v>3000</v>
       </c>
@@ -7877,7 +7877,7 @@
       </c>
       <c r="S70" s="28"/>
     </row>
-    <row r="71" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A71" s="16">
         <v>0</v>
       </c>
@@ -7933,7 +7933,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="72" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A72" s="16">
         <v>0</v>
       </c>
@@ -7992,7 +7992,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="73" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A73" s="16">
         <v>0</v>
       </c>
@@ -8051,7 +8051,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
         <v>78</v>
       </c>
@@ -8106,7 +8106,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A75" s="10" t="s">
         <v>79</v>
       </c>
@@ -8161,7 +8161,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
         <v>80</v>
       </c>
@@ -8216,7 +8216,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>7009</v>
       </c>
@@ -8272,7 +8272,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>7008</v>
       </c>
@@ -8325,7 +8325,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>9388</v>
       </c>
@@ -8378,7 +8378,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>9389</v>
       </c>
@@ -8431,7 +8431,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>9300</v>
       </c>
@@ -8485,7 +8485,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>0</v>
       </c>
@@ -8538,12 +8538,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A84" s="10">
         <f>IF(LEN(C84)=17,LEFT(C84,4)+(B84-1)/(DATE(LEFT(C84,4)+1,1,1)-DATE(LEFT(C84,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2021.4958923135464</v>
@@ -8565,7 +8565,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A85" s="35">
         <v>1000</v>
       </c>
@@ -8623,7 +8623,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A86" s="16">
         <v>2010</v>
       </c>
@@ -8679,7 +8679,7 @@
       </c>
       <c r="S86" s="28"/>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A87" s="35">
         <v>3000</v>
       </c>
@@ -8737,7 +8737,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="88" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A88" s="35">
         <v>0</v>
       </c>
@@ -8790,7 +8790,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="89" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A89" s="16">
         <v>0</v>
       </c>
@@ -8843,7 +8843,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="90" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A90" s="35">
         <v>0</v>
       </c>
@@ -8896,7 +8896,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A91" s="36" t="s">
         <v>78</v>
       </c>
@@ -8952,7 +8952,7 @@
       </c>
       <c r="S91" s="28"/>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A92" s="10" t="s">
         <v>79</v>
       </c>
@@ -9008,7 +9008,7 @@
       </c>
       <c r="S92" s="28"/>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A93" s="36" t="s">
         <v>80</v>
       </c>
@@ -9064,7 +9064,7 @@
       </c>
       <c r="S93" s="28"/>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>9300</v>
       </c>
@@ -9118,7 +9118,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A95" s="25">
         <v>9380</v>
       </c>
@@ -9171,7 +9171,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A96" s="25">
         <v>9381</v>
       </c>
@@ -9224,7 +9224,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>0</v>
       </c>
@@ -9277,12 +9277,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A99" s="10">
         <f>IF(LEN(C99)=17,LEFT(C99,4)+(B99-1)/(DATE(LEFT(C99,4)+1,1,1)-DATE(LEFT(C99,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2022.5466628614915</v>
@@ -9301,7 +9301,7 @@
       <c r="P99" s="48"/>
       <c r="Q99" s="48"/>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A100" s="16">
         <v>1000</v>
       </c>
@@ -9357,7 +9357,7 @@
       </c>
       <c r="S100" s="28"/>
     </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A101" s="16">
         <v>2010</v>
       </c>
@@ -9413,7 +9413,7 @@
       </c>
       <c r="S101" s="28"/>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A102" s="16">
         <v>3000</v>
       </c>
@@ -9469,7 +9469,7 @@
       </c>
       <c r="S102" s="28"/>
     </row>
-    <row r="103" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A103" s="16">
         <v>0</v>
       </c>
@@ -9522,7 +9522,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="104" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A104" s="16">
         <v>0</v>
       </c>
@@ -9575,7 +9575,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="105" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A105" s="16">
         <v>0</v>
       </c>
@@ -9628,7 +9628,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A106" s="10" t="s">
         <v>78</v>
       </c>
@@ -9684,7 +9684,7 @@
       </c>
       <c r="S106" s="28"/>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A107" s="10" t="s">
         <v>79</v>
       </c>
@@ -9740,7 +9740,7 @@
       </c>
       <c r="S107" s="28"/>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A108" s="10" t="s">
         <v>80</v>
       </c>
@@ -9796,7 +9796,7 @@
       </c>
       <c r="S108" s="28"/>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>9300</v>
       </c>
@@ -9845,7 +9845,7 @@
       </c>
       <c r="Q109" s="48"/>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>9380</v>
       </c>
@@ -9891,7 +9891,7 @@
       <c r="P110" s="48"/>
       <c r="Q110" s="48"/>
     </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>9381</v>
       </c>
@@ -9937,7 +9937,7 @@
       <c r="P111" s="48"/>
       <c r="Q111" s="48"/>
     </row>
-    <row r="112" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>0</v>
       </c>
@@ -9990,12 +9990,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="114" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A114" s="10">
         <f>IF(LEN(C114)=17,LEFT(C114,4)+(B114-1)/(DATE(LEFT(C114,4)+1,1,1)-DATE(LEFT(C114,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2024.084701350941</v>
@@ -10014,7 +10014,7 @@
       <c r="P114" s="48"/>
       <c r="Q114" s="48"/>
     </row>
-    <row r="115" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>0</v>
       </c>
@@ -10067,7 +10067,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="116" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>0</v>
       </c>
@@ -10120,7 +10120,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="117" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A117" s="16">
         <v>1000</v>
       </c>
@@ -10176,7 +10176,7 @@
       </c>
       <c r="S117" s="28"/>
     </row>
-    <row r="118" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A118" s="16">
         <v>0</v>
       </c>
@@ -10230,7 +10230,7 @@
       </c>
       <c r="S118" s="28"/>
     </row>
-    <row r="119" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A119" s="16">
         <v>0</v>
       </c>
@@ -10288,7 +10288,7 @@
       </c>
       <c r="S119" s="28"/>
     </row>
-    <row r="120" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A120" s="35">
         <v>0</v>
       </c>
@@ -10342,7 +10342,7 @@
       </c>
       <c r="S120" s="28"/>
     </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A121" s="16">
         <v>2010</v>
       </c>
@@ -10398,7 +10398,7 @@
       </c>
       <c r="S121" s="28"/>
     </row>
-    <row r="122" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A122" s="16">
         <v>0</v>
       </c>
@@ -10452,7 +10452,7 @@
       </c>
       <c r="S122" s="28"/>
     </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A123" s="16">
         <v>0</v>
       </c>
@@ -10510,7 +10510,7 @@
       </c>
       <c r="S123" s="28"/>
     </row>
-    <row r="124" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A124" s="35">
         <v>0</v>
       </c>
@@ -10564,7 +10564,7 @@
       </c>
       <c r="S124" s="28"/>
     </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A125" s="16">
         <v>3000</v>
       </c>
@@ -10620,7 +10620,7 @@
       </c>
       <c r="S125" s="28"/>
     </row>
-    <row r="126" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A126" s="16">
         <v>0</v>
       </c>
@@ -10673,7 +10673,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A127" s="16">
         <v>0</v>
       </c>
@@ -10730,7 +10730,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="128" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A128" s="25">
         <v>0</v>
       </c>
@@ -10783,7 +10783,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="129" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A129" s="25">
         <v>0</v>
       </c>
@@ -10837,7 +10837,7 @@
       </c>
       <c r="S129" s="28"/>
     </row>
-    <row r="130" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>9300</v>
       </c>
@@ -10891,7 +10891,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="131" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>0</v>
       </c>
@@ -10944,7 +10944,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="132" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>0</v>
       </c>
@@ -10998,7 +10998,7 @@
       </c>
       <c r="S132" s="28"/>
     </row>
-    <row r="133" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>0</v>
       </c>
@@ -11051,7 +11051,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="134" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A134" s="47">
         <v>0</v>
       </c>
@@ -11104,7 +11104,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="135" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A135" s="47">
         <v>0</v>
       </c>
@@ -11157,7 +11157,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="136" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>0</v>
       </c>
@@ -11210,7 +11210,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="137" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>0</v>
       </c>
@@ -11263,12 +11263,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="138" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="139" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A139" s="10">
         <f>IF(LEN(C139)=17,LEFT(C139,4)+(B139-1)/(DATE(LEFT(C139,4)+1,1,1)-DATE(LEFT(C139,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2024.5819691105039</v>
@@ -11287,7 +11287,7 @@
       <c r="P139" s="48"/>
       <c r="Q139" s="48"/>
     </row>
-    <row r="140" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>0</v>
       </c>
@@ -11340,7 +11340,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="141" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>0</v>
       </c>
@@ -11393,7 +11393,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="142" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>1000</v>
       </c>
@@ -11450,7 +11450,7 @@
       </c>
       <c r="S142" s="28"/>
     </row>
-    <row r="143" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>0</v>
       </c>
@@ -11504,7 +11504,7 @@
       </c>
       <c r="S143" s="28"/>
     </row>
-    <row r="144" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>0</v>
       </c>
@@ -11562,7 +11562,7 @@
       </c>
       <c r="S144" s="28"/>
     </row>
-    <row r="145" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>0</v>
       </c>
@@ -11616,7 +11616,7 @@
       </c>
       <c r="S145" s="28"/>
     </row>
-    <row r="146" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>2010</v>
       </c>
@@ -11673,7 +11673,7 @@
       </c>
       <c r="S146" s="28"/>
     </row>
-    <row r="147" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>0</v>
       </c>
@@ -11727,7 +11727,7 @@
       </c>
       <c r="S147" s="28"/>
     </row>
-    <row r="148" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>0</v>
       </c>
@@ -11785,7 +11785,7 @@
       </c>
       <c r="S148" s="28"/>
     </row>
-    <row r="149" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>0</v>
       </c>
@@ -11839,7 +11839,7 @@
       </c>
       <c r="S149" s="28"/>
     </row>
-    <row r="150" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>3000</v>
       </c>
@@ -11896,7 +11896,7 @@
       </c>
       <c r="S150" s="28"/>
     </row>
-    <row r="151" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>0</v>
       </c>
@@ -11949,7 +11949,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="152" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>0</v>
       </c>
@@ -12006,7 +12006,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="153" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>0</v>
       </c>
@@ -12059,7 +12059,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="154" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>0</v>
       </c>
@@ -12113,7 +12113,7 @@
       </c>
       <c r="S154" s="28"/>
     </row>
-    <row r="155" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>9300</v>
       </c>
@@ -12167,7 +12167,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="156" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>0</v>
       </c>
@@ -12220,7 +12220,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="157" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>0</v>
       </c>
@@ -12274,7 +12274,7 @@
       </c>
       <c r="S157" s="28"/>
     </row>
-    <row r="158" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>0</v>
       </c>
@@ -12327,7 +12327,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="159" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>0</v>
       </c>
@@ -12380,7 +12380,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="160" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>0</v>
       </c>
@@ -12433,12 +12433,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="161" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="162" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A162" s="10">
         <f>IF(LEN(C162)=17,LEFT(C162,4)+(B162-1)/(DATE(LEFT(C162,4)+1,1,1)-DATE(LEFT(C162,4),1,1)),"BAD DATE FORMAT")</f>
         <v>2025.5808238203958</v>
@@ -12457,7 +12457,7 @@
       <c r="P162" s="48"/>
       <c r="Q162" s="48"/>
     </row>
-    <row r="163" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>0</v>
       </c>
@@ -12514,7 +12514,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="164" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>0</v>
       </c>
@@ -12572,7 +12572,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="165" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>0</v>
       </c>
@@ -12633,7 +12633,7 @@
       </c>
       <c r="S165" s="28"/>
     </row>
-    <row r="166" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A166" s="25">
         <v>1000</v>
       </c>
@@ -12694,7 +12694,7 @@
       </c>
       <c r="S166" s="28"/>
     </row>
-    <row r="167" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>0</v>
       </c>
@@ -12755,7 +12755,7 @@
       </c>
       <c r="S167" s="28"/>
     </row>
-    <row r="168" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>0</v>
       </c>
@@ -12816,7 +12816,7 @@
       </c>
       <c r="S168" s="28"/>
     </row>
-    <row r="169" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>0</v>
       </c>
@@ -12877,7 +12877,7 @@
       </c>
       <c r="S169" s="28"/>
     </row>
-    <row r="170" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A170" s="25">
         <v>2010</v>
       </c>
@@ -12938,7 +12938,7 @@
       </c>
       <c r="S170" s="28"/>
     </row>
-    <row r="171" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>0</v>
       </c>
@@ -12999,7 +12999,7 @@
       </c>
       <c r="S171" s="28"/>
     </row>
-    <row r="172" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>0</v>
       </c>
@@ -13060,7 +13060,7 @@
       </c>
       <c r="S172" s="28"/>
     </row>
-    <row r="173" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>0</v>
       </c>
@@ -13121,7 +13121,7 @@
       </c>
       <c r="S173" s="28"/>
     </row>
-    <row r="174" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A174" s="25">
         <v>3000</v>
       </c>
@@ -13181,7 +13181,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="175" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>0</v>
       </c>
@@ -13241,7 +13241,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="176" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>0</v>
       </c>
@@ -13301,7 +13301,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="177" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>0</v>
       </c>
@@ -13360,7 +13360,7 @@
       </c>
       <c r="S177" s="28"/>
     </row>
-    <row r="178" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>9300</v>
       </c>
@@ -13419,7 +13419,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="179" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>0</v>
       </c>
@@ -13477,7 +13477,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="180" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>0</v>
       </c>
@@ -13536,7 +13536,7 @@
       </c>
       <c r="S180" s="28"/>
     </row>
-    <row r="181" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>0</v>
       </c>
@@ -13594,7 +13594,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="182" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>0</v>
       </c>
@@ -13652,7 +13652,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="183" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>0</v>
       </c>
@@ -13710,7 +13710,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="184" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A184" s="25">
         <v>0</v>
       </c>
@@ -13766,7 +13766,7 @@
         <v>R = 1000/M</v>
       </c>
     </row>
-    <row r="185" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A185" s="25">
         <v>0</v>
       </c>
@@ -13837,12 +13837,12 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA7BD733-D02F-4818-9D6A-E6E21FE780ED}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.6640625" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="71" t="s">
         <v>256</v>
       </c>
@@ -13868,7 +13868,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="54" t="s">
         <v>257</v>
       </c>
@@ -13878,8 +13878,11 @@
       <c r="C2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="54" t="s">
         <v>258</v>
       </c>
@@ -13889,8 +13892,11 @@
       <c r="C3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="54" t="s">
         <v>259</v>
       </c>
@@ -13900,8 +13906,11 @@
       <c r="C4">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="54" t="s">
         <v>260</v>
       </c>
@@ -13911,8 +13920,11 @@
       <c r="C5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="54" t="s">
         <v>261</v>
       </c>
@@ -13922,8 +13934,11 @@
       <c r="C6">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="54" t="s">
         <v>262</v>
       </c>
@@ -13933,8 +13948,11 @@
       <c r="C7">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="54" t="s">
         <v>263</v>
       </c>
@@ -13944,8 +13962,11 @@
       <c r="C8">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="54" t="s">
         <v>271</v>
       </c>
@@ -13958,11 +13979,14 @@
       <c r="D9">
         <v>3</v>
       </c>
+      <c r="E9">
+        <v>14</v>
+      </c>
       <c r="F9">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="54" t="s">
         <v>264</v>
       </c>
@@ -13982,7 +14006,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="54" t="s">
         <v>265</v>
       </c>
@@ -13999,7 +14023,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="54" t="s">
         <v>266</v>
       </c>
@@ -14016,7 +14040,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="54" t="s">
         <v>267</v>
       </c>
@@ -14039,7 +14063,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="54" t="s">
         <v>268</v>
       </c>
@@ -14062,7 +14086,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="54" t="s">
         <v>269</v>
       </c>
@@ -14093,22 +14117,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B5CE66C-33D7-49A1-8DF7-7981795B80E7}">
   <dimension ref="A1:P147"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="8" max="8" width="29.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>200</v>
       </c>
@@ -14158,7 +14182,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>122</v>
       </c>
@@ -14187,7 +14211,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>123</v>
       </c>
@@ -14216,7 +14240,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>124</v>
       </c>
@@ -14251,7 +14275,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>125</v>
       </c>
@@ -14298,7 +14322,7 @@
         <v>1.7168308506891199</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>126</v>
       </c>
@@ -14333,7 +14357,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>127</v>
       </c>
@@ -14368,7 +14392,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>128</v>
       </c>
@@ -14403,7 +14427,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>129</v>
       </c>
@@ -14450,7 +14474,7 @@
         <v>1.0501569268589599</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>130</v>
       </c>
@@ -14485,7 +14509,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>131</v>
       </c>
@@ -14520,7 +14544,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>132</v>
       </c>
@@ -14555,7 +14579,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>133</v>
       </c>
@@ -14602,7 +14626,7 @@
         <v>0.94600494833357596</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>134</v>
       </c>
@@ -14637,7 +14661,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>135</v>
       </c>
@@ -14672,7 +14696,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>136</v>
       </c>
@@ -14701,7 +14725,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>137</v>
       </c>
@@ -14748,7 +14772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>138</v>
       </c>
@@ -14774,7 +14798,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>139</v>
       </c>
@@ -14800,7 +14824,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>140</v>
       </c>
@@ -14826,7 +14850,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>141</v>
       </c>
@@ -14855,7 +14879,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>142</v>
       </c>
@@ -14884,7 +14908,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>143</v>
       </c>
@@ -14925,7 +14949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>144</v>
       </c>
@@ -14966,7 +14990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>78</v>
       </c>
@@ -14995,7 +15019,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>79</v>
       </c>
@@ -15024,7 +15048,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>80</v>
       </c>
@@ -15071,7 +15095,7 @@
         <v>1.2587336487582701</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>81</v>
       </c>
@@ -15106,7 +15130,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>82</v>
       </c>
@@ -15156,7 +15180,7 @@
         <v>1.2587336487582701</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>83</v>
       </c>
@@ -15191,7 +15215,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>84</v>
       </c>
@@ -15238,7 +15262,7 @@
         <v>1.8811551773110999</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>85</v>
       </c>
@@ -15273,7 +15297,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>86</v>
       </c>
@@ -15323,7 +15347,7 @@
         <v>1.8811551773110999</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>87</v>
       </c>
@@ -15358,7 +15382,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>88</v>
       </c>
@@ -15405,7 +15429,7 @@
         <v>1.2914628942617901</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>89</v>
       </c>
@@ -15440,7 +15464,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>90</v>
       </c>
@@ -15490,7 +15514,7 @@
         <v>1.2914628942617901</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>91</v>
       </c>
@@ -15525,7 +15549,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>92</v>
       </c>
@@ -15554,7 +15578,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>93</v>
       </c>
@@ -15601,7 +15625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>94</v>
       </c>
@@ -15627,7 +15651,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>95</v>
       </c>
@@ -15653,7 +15677,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>96</v>
       </c>
@@ -15679,7 +15703,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>97</v>
       </c>
@@ -15714,7 +15738,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>98</v>
       </c>
@@ -15749,7 +15773,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>99</v>
       </c>
@@ -15784,7 +15808,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>100</v>
       </c>
@@ -15819,7 +15843,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>101</v>
       </c>
@@ -15848,7 +15872,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>102</v>
       </c>
@@ -15877,7 +15901,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>103</v>
       </c>
@@ -15921,7 +15945,7 @@
         <v>2.52101822944072</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>104</v>
       </c>
@@ -15953,7 +15977,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>105</v>
       </c>
@@ -16000,7 +16024,7 @@
         <v>2.52101822944072</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>106</v>
       </c>
@@ -16032,7 +16056,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>107</v>
       </c>
@@ -16079,7 +16103,7 @@
         <v>0.929754688179387</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>108</v>
       </c>
@@ -16114,7 +16138,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>109</v>
       </c>
@@ -16164,7 +16188,7 @@
         <v>0.929754688179387</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>110</v>
       </c>
@@ -16199,7 +16223,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>111</v>
       </c>
@@ -16246,7 +16270,7 @@
         <v>2.4150196263511101</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>112</v>
       </c>
@@ -16281,7 +16305,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>113</v>
       </c>
@@ -16331,7 +16355,7 @@
         <v>2.4150196263511101</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>114</v>
       </c>
@@ -16366,7 +16390,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>115</v>
       </c>
@@ -16395,7 +16419,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>116</v>
       </c>
@@ -16442,7 +16466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>117</v>
       </c>
@@ -16468,7 +16492,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>118</v>
       </c>
@@ -16494,7 +16518,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>119</v>
       </c>
@@ -16520,7 +16544,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>120</v>
       </c>
@@ -16549,7 +16573,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>121</v>
       </c>
@@ -16578,7 +16602,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>65</v>
       </c>
@@ -16625,7 +16649,7 @@
         <v>1.16405016530411</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>66</v>
       </c>
@@ -16672,7 +16696,7 @@
         <v>1.8352099609999999</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>67</v>
       </c>
@@ -16719,7 +16743,7 @@
         <v>1.2169603471391199</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>68</v>
       </c>
@@ -16754,7 +16778,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>69</v>
       </c>
@@ -16789,7 +16813,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>70</v>
       </c>
@@ -16824,7 +16848,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>71</v>
       </c>
@@ -16874,7 +16898,7 @@
         <v>1.16405016530411</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>72</v>
       </c>
@@ -16924,7 +16948,7 @@
         <v>1.8352099609999999</v>
       </c>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>73</v>
       </c>
@@ -16974,7 +16998,7 @@
         <v>1.2169603471391199</v>
       </c>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>74</v>
       </c>
@@ -17021,7 +17045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>75</v>
       </c>
@@ -17071,7 +17095,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>76</v>
       </c>
@@ -17121,7 +17145,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>77</v>
       </c>
@@ -17147,7 +17171,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>37</v>
       </c>
@@ -17194,7 +17218,7 @@
         <v>1.80205774681044</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>38</v>
       </c>
@@ -17241,7 +17265,7 @@
         <v>2.03531169831321</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>39</v>
       </c>
@@ -17288,7 +17312,7 @@
         <v>2.20773173146471</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>40</v>
       </c>
@@ -17320,7 +17344,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>41</v>
       </c>
@@ -17352,7 +17376,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>42</v>
       </c>
@@ -17384,7 +17408,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>43</v>
       </c>
@@ -17434,7 +17458,7 @@
         <v>1.80205774681044</v>
       </c>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>44</v>
       </c>
@@ -17484,7 +17508,7 @@
         <v>2.03531169831321</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>45</v>
       </c>
@@ -17534,7 +17558,7 @@
         <v>2.20773173146471</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>46</v>
       </c>
@@ -17581,7 +17605,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>47</v>
       </c>
@@ -17628,7 +17652,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>48</v>
       </c>
@@ -17675,7 +17699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>49</v>
       </c>
@@ -17722,7 +17746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>50</v>
       </c>
@@ -17769,7 +17793,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>51</v>
       </c>
@@ -17795,7 +17819,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>52</v>
       </c>
@@ -17842,7 +17866,7 @@
         <v>0.76827735566056199</v>
       </c>
     </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>53</v>
       </c>
@@ -17889,7 +17913,7 @@
         <v>2.03531169831321</v>
       </c>
     </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>54</v>
       </c>
@@ -17936,7 +17960,7 @@
         <v>0.83122061412608705</v>
       </c>
     </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>55</v>
       </c>
@@ -17971,7 +17995,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>56</v>
       </c>
@@ -18006,7 +18030,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>57</v>
       </c>
@@ -18041,7 +18065,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>58</v>
       </c>
@@ -18091,7 +18115,7 @@
         <v>0.76827735566056199</v>
       </c>
     </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>59</v>
       </c>
@@ -18141,7 +18165,7 @@
         <v>2.03531169831321</v>
       </c>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>60</v>
       </c>
@@ -18191,7 +18215,7 @@
         <v>0.83122061412608705</v>
       </c>
     </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>61</v>
       </c>
@@ -18238,7 +18262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>62</v>
       </c>
@@ -18288,7 +18312,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>63</v>
       </c>
@@ -18338,7 +18362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>64</v>
       </c>
@@ -18364,7 +18388,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>18</v>
       </c>
@@ -18411,7 +18435,7 @@
         <v>1.67449813656697</v>
       </c>
     </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>19</v>
       </c>
@@ -18458,7 +18482,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>20</v>
       </c>
@@ -18502,7 +18526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>21</v>
       </c>
@@ -18528,7 +18552,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>22</v>
       </c>
@@ -18575,7 +18599,7 @@
         <v>1.67449813656697</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>23</v>
       </c>
@@ -18622,7 +18646,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>24</v>
       </c>
@@ -18669,7 +18693,7 @@
         <v>2.2908047722416698</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>25</v>
       </c>
@@ -18701,7 +18725,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>26</v>
       </c>
@@ -18733,7 +18757,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>27</v>
       </c>
@@ -18765,7 +18789,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>28</v>
       </c>
@@ -18812,7 +18836,7 @@
         <v>1.67449813656697</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>28.5</v>
       </c>
@@ -18859,7 +18883,7 @@
         <v>2.2908047722416698</v>
       </c>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>29</v>
       </c>
@@ -18906,7 +18930,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>30</v>
       </c>
@@ -18953,7 +18977,7 @@
         <v>2.2908047722416698</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>31</v>
       </c>
@@ -19000,7 +19024,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>32</v>
       </c>
@@ -19047,7 +19071,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>33</v>
       </c>
@@ -19094,7 +19118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>34</v>
       </c>
@@ -19141,7 +19165,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>35</v>
       </c>
@@ -19185,7 +19209,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>36</v>
       </c>
@@ -19211,7 +19235,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>15</v>
       </c>
@@ -19258,7 +19282,7 @@
         <v>1.67262493287749</v>
       </c>
     </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>16</v>
       </c>
@@ -19305,7 +19329,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>17</v>
       </c>
@@ -19349,7 +19373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>12</v>
       </c>
@@ -19396,7 +19420,7 @@
         <v>1.67075591548251</v>
       </c>
     </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>13</v>
       </c>
@@ -19443,7 +19467,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>14</v>
       </c>
@@ -19487,7 +19511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>6</v>
       </c>
@@ -19534,7 +19558,7 @@
         <v>1.6226717989921</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>7</v>
       </c>
@@ -19581,7 +19605,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>8</v>
       </c>
@@ -19625,7 +19649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>9</v>
       </c>
@@ -19672,7 +19696,7 @@
         <v>1.66982297226244</v>
       </c>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>10</v>
       </c>
@@ -19719,7 +19743,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>11</v>
       </c>
@@ -19763,7 +19787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>3</v>
       </c>
@@ -19810,7 +19834,7 @@
         <v>1.6188010157323101</v>
       </c>
     </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>4</v>
       </c>
@@ -19857,7 +19881,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>5</v>
       </c>
@@ -19901,7 +19925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>0</v>
       </c>
@@ -19949,7 +19973,7 @@
         <v>1.6168725409881399</v>
       </c>
     </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>1</v>
       </c>
@@ -19996,7 +20020,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="147" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>2</v>
       </c>
@@ -20051,20 +20075,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C2AC3CD-B28B-4E07-84D1-63F10D71EFF6}">
   <dimension ref="A1:O14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="14.5" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="14.5" customWidth="1"/>
-    <col min="13" max="13" width="13.5" customWidth="1"/>
-    <col min="14" max="14" width="15.33203125" customWidth="1"/>
-    <col min="15" max="15" width="13.5" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" customWidth="1"/>
+    <col min="13" max="13" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="15.28515625" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="60" t="s">
         <v>201</v>
       </c>
@@ -20111,7 +20135,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="57">
         <v>2015</v>
       </c>
@@ -20158,7 +20182,7 @@
         <v>1.6168725409881399</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="56">
         <v>2016</v>
       </c>
@@ -20205,7 +20229,7 @@
         <v>1.6188010157323101</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="56">
         <v>2017</v>
       </c>
@@ -20252,7 +20276,7 @@
         <v>1.6226717989921</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="57">
         <v>2017</v>
       </c>
@@ -20299,7 +20323,7 @@
         <v>1.66982297226244</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="57">
         <v>2018</v>
       </c>
@@ -20346,7 +20370,7 @@
         <v>1.67075591548251</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="56">
         <v>2019</v>
       </c>
@@ -20393,7 +20417,7 @@
         <v>1.67262493287749</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="56">
         <v>2020</v>
       </c>
@@ -20440,7 +20464,7 @@
         <v>1.67449813656697</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="57">
         <v>2020</v>
       </c>
@@ -20487,7 +20511,7 @@
         <v>1.67449813656697</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="56">
         <v>2021</v>
       </c>
@@ -20534,7 +20558,7 @@
         <v>1.80205774681044</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="56">
         <v>2021</v>
       </c>
@@ -20581,7 +20605,7 @@
         <v>0.76827735566056199</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="56">
         <v>2022</v>
       </c>
@@ -20628,7 +20652,7 @@
         <v>1.16405016530411</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="57">
         <v>2024</v>
       </c>
@@ -20675,7 +20699,7 @@
         <v>1.2587336487582701</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="57">
         <v>2025</v>
       </c>
@@ -20734,20 +20758,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D50481-F00D-4F48-81C6-07265F307B30}">
   <dimension ref="A1:O15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="14.5" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="14.5" customWidth="1"/>
-    <col min="13" max="13" width="13.5" customWidth="1"/>
-    <col min="14" max="14" width="15.33203125" customWidth="1"/>
-    <col min="15" max="15" width="13.5" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" customWidth="1"/>
+    <col min="13" max="13" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="15.28515625" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="62" t="s">
         <v>201</v>
       </c>
@@ -20794,7 +20818,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="63">
         <v>2015</v>
       </c>
@@ -20839,7 +20863,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="64">
         <v>2016</v>
       </c>
@@ -20884,7 +20908,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="63">
         <v>2017</v>
       </c>
@@ -20929,7 +20953,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="64">
         <v>2017</v>
       </c>
@@ -20974,7 +20998,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="63">
         <v>2018</v>
       </c>
@@ -21019,7 +21043,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="64">
         <v>2019</v>
       </c>
@@ -21064,7 +21088,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="63">
         <v>2020</v>
       </c>
@@ -21109,7 +21133,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="64">
         <v>2020</v>
       </c>
@@ -21154,7 +21178,7 @@
         <v>1.9286659923145</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="69">
         <v>2021</v>
       </c>
@@ -21199,7 +21223,7 @@
         <v>2.03531169831321</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="72">
         <v>2021</v>
       </c>
@@ -21244,7 +21268,7 @@
         <v>2.03531169831321</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="74">
         <v>2022</v>
       </c>
@@ -21289,7 +21313,7 @@
         <v>1.8352099609999999</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="74">
         <v>2024</v>
       </c>
@@ -21334,7 +21358,7 @@
         <v>1.8811551773110999</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="72">
         <v>2024</v>
       </c>
@@ -21379,7 +21403,7 @@
         <v>0.929754688179387</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="74">
         <v>2025</v>
       </c>
@@ -21422,7 +21446,7 @@
       <c r="N15" s="64">
         <v>119.336014415791</v>
       </c>
-      <c r="O15" s="80">
+      <c r="O15" s="76">
         <v>1.0501569268589599</v>
       </c>
     </row>
@@ -21437,20 +21461,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71D78007-B334-4AFA-9368-61BFA621700B}">
   <dimension ref="A1:O8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="14.5" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="14.5" customWidth="1"/>
-    <col min="13" max="13" width="13.5" customWidth="1"/>
-    <col min="14" max="14" width="15.33203125" customWidth="1"/>
-    <col min="15" max="15" width="13.5" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" customWidth="1"/>
+    <col min="13" max="13" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="15.28515625" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="62" t="s">
         <v>201</v>
       </c>
@@ -21497,7 +21521,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="63">
         <v>2020</v>
       </c>
@@ -21542,7 +21566,7 @@
         <v>2.2908047722416698</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="64">
         <v>2021</v>
       </c>
@@ -21587,7 +21611,7 @@
         <v>2.20773173146471</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="63">
         <v>2021</v>
       </c>
@@ -21632,7 +21656,7 @@
         <v>0.83122061412608705</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="64">
         <v>2022</v>
       </c>
@@ -21677,7 +21701,7 @@
         <v>1.2169603471391199</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="64">
         <v>2024</v>
       </c>
@@ -21722,7 +21746,7 @@
         <v>1.2914628942617901</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="69">
         <v>2024</v>
       </c>
@@ -21767,7 +21791,7 @@
         <v>2.4150196263511101</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="67">
         <v>2025</v>
       </c>
@@ -21823,20 +21847,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EB1D8E7-B939-4F56-8304-C86C81BE8A5F}">
   <dimension ref="A1:O7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="14.5" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="14.5" customWidth="1"/>
-    <col min="13" max="13" width="13.5" customWidth="1"/>
-    <col min="14" max="14" width="15.33203125" customWidth="1"/>
-    <col min="15" max="15" width="13.5" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" customWidth="1"/>
+    <col min="13" max="13" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="15.28515625" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="62" t="s">
         <v>201</v>
       </c>
@@ -21883,7 +21907,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="63">
         <v>2025</v>
       </c>
@@ -21928,7 +21952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="64">
         <v>2024</v>
       </c>
@@ -21973,7 +21997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="63">
         <v>2024</v>
       </c>
@@ -22018,7 +22042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="64">
         <v>2022</v>
       </c>
@@ -22063,7 +22087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="63">
         <v>2021</v>
       </c>
@@ -22108,7 +22132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="67">
         <v>2021</v>
       </c>
@@ -22164,20 +22188,20 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1159179F-CF4E-4E88-AA90-1605119874FB}">
   <dimension ref="A1:O15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="14.5" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="14.5" customWidth="1"/>
-    <col min="13" max="13" width="13.5" customWidth="1"/>
-    <col min="14" max="14" width="15.33203125" customWidth="1"/>
-    <col min="15" max="15" width="13.5" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" customWidth="1"/>
+    <col min="13" max="13" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="15.28515625" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="62" t="s">
         <v>201</v>
       </c>
@@ -22224,7 +22248,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="63">
         <v>2021</v>
       </c>
@@ -22259,7 +22283,7 @@
       <c r="N2" s="63"/>
       <c r="O2" s="63"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="64">
         <v>2021</v>
       </c>
@@ -22294,7 +22318,7 @@
       <c r="N3" s="64"/>
       <c r="O3" s="64"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="63">
         <v>2021</v>
       </c>
@@ -22329,7 +22353,7 @@
       <c r="N4" s="63"/>
       <c r="O4" s="63"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="64">
         <v>2021</v>
       </c>
@@ -22374,7 +22398,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="63">
         <v>2021</v>
       </c>
@@ -22419,7 +22443,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="64">
         <v>2021</v>
       </c>
@@ -22464,7 +22488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="63">
         <v>2021</v>
       </c>
@@ -22509,7 +22533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="64">
         <v>2020</v>
       </c>
@@ -22544,7 +22568,7 @@
       <c r="N9" s="64"/>
       <c r="O9" s="64"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="63">
         <v>2020</v>
       </c>
@@ -22579,7 +22603,7 @@
       <c r="N10" s="63"/>
       <c r="O10" s="63"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="64">
         <v>2020</v>
       </c>
@@ -22614,7 +22638,7 @@
       <c r="N11" s="64"/>
       <c r="O11" s="64"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="63">
         <v>2020</v>
       </c>
@@ -22659,7 +22683,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="64">
         <v>2020</v>
       </c>
@@ -22704,7 +22728,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="63">
         <v>2020</v>
       </c>
@@ -22749,7 +22773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="67">
         <v>2020</v>
       </c>
@@ -22805,20 +22829,20 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7847FC27-2935-424C-A158-6B9B5A8DB710}">
   <dimension ref="A1:O4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="14.5" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="14.5" customWidth="1"/>
-    <col min="13" max="13" width="13.5" customWidth="1"/>
-    <col min="14" max="14" width="15.33203125" customWidth="1"/>
-    <col min="15" max="15" width="13.5" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" customWidth="1"/>
+    <col min="13" max="13" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="15.28515625" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="62" t="s">
         <v>201</v>
       </c>
@@ -22865,7 +22889,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="63">
         <v>2025</v>
       </c>
@@ -22900,7 +22924,7 @@
       <c r="N2" s="63"/>
       <c r="O2" s="63"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="64">
         <v>2024</v>
       </c>
@@ -22935,7 +22959,7 @@
       <c r="N3" s="64"/>
       <c r="O3" s="64"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="69">
         <v>2024</v>
       </c>
@@ -22981,20 +23005,20 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC7BE515-81CD-497C-A39A-B15BC3D309FD}">
   <dimension ref="A1:O4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="14.5" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="14.5" customWidth="1"/>
-    <col min="13" max="13" width="13.5" customWidth="1"/>
-    <col min="14" max="14" width="15.33203125" customWidth="1"/>
-    <col min="15" max="15" width="13.5" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" customWidth="1"/>
+    <col min="13" max="13" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="15.28515625" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="62" t="s">
         <v>201</v>
       </c>
@@ -23041,7 +23065,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="63">
         <v>2025</v>
       </c>
@@ -23076,7 +23100,7 @@
       <c r="N2" s="63"/>
       <c r="O2" s="63"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="64">
         <v>2024</v>
       </c>
@@ -23111,7 +23135,7 @@
       <c r="N3" s="64"/>
       <c r="O3" s="64"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="69">
         <v>2024</v>
       </c>

</xml_diff>